<commit_message>
CI Reports [2026-06-29 18:11]: ActionQueue — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/ActionQueue.xlsx
+++ b/Test Execution Report_Git/Feature Reports/ActionQueue.xlsx
@@ -500,7 +500,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K2" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="L2" t="str">
         <v>FAIL</v>
@@ -550,7 +550,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K3" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="L3" t="str">
         <v>FAIL</v>
@@ -600,7 +600,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K4" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="L4" t="str">
         <v>FAIL</v>
@@ -650,7 +650,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K5" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="L5" t="str">
         <v>FAIL</v>
@@ -700,7 +700,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K6" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="L6" t="str">
         <v>FAIL</v>
@@ -750,7 +750,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K7" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="L7" t="str">
         <v>FAIL</v>
@@ -800,7 +800,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K8" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="L8" t="str">
         <v>FAIL</v>
@@ -900,7 +900,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K10" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="L10" t="str">
         <v>FAIL</v>
@@ -950,7 +950,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K11" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L11" t="str">
         <v>FAIL</v>
@@ -1050,7 +1050,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K13" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L13" t="str">
         <v>FAIL</v>
@@ -1100,7 +1100,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K14" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L14" t="str">
         <v>FAIL</v>
@@ -1150,7 +1150,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K15" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L15" t="str">
         <v>FAIL</v>
@@ -1200,7 +1200,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K16" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L16" t="str">
         <v>FAIL</v>
@@ -1250,7 +1250,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K17" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L17" t="str">
         <v>FAIL</v>
@@ -1300,7 +1300,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K18" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L18" t="str">
         <v>FAIL</v>
@@ -1350,7 +1350,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K19" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L19" t="str">
         <v>FAIL</v>
@@ -1400,7 +1400,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K20" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L20" t="str">
         <v>FAIL</v>
@@ -1450,7 +1450,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K21" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L21" t="str">
         <v>FAIL</v>
@@ -1500,7 +1500,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K22" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L22" t="str">
         <v>FAIL</v>
@@ -1550,7 +1550,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K23" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L23" t="str">
         <v>FAIL</v>
@@ -1600,7 +1600,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K24" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L24" t="str">
         <v>FAIL</v>
@@ -1650,7 +1650,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K25" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L25" t="str">
         <v>FAIL</v>
@@ -1700,7 +1700,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K26" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L26" t="str">
         <v>FAIL</v>
@@ -1750,7 +1750,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K27" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="L27" t="str">
         <v>FAIL</v>
@@ -1877,7 +1877,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J2" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="K2" t="str">
         <v>New</v>
@@ -1928,7 +1928,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J3" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="K3" t="str">
         <v>New</v>
@@ -1979,7 +1979,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J4" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="K4" t="str">
         <v>New</v>
@@ -2030,7 +2030,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J5" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="K5" t="str">
         <v>New</v>
@@ -2081,7 +2081,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J6" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="K6" t="str">
         <v>New</v>
@@ -2132,7 +2132,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J7" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="K7" t="str">
         <v>New</v>
@@ -2183,7 +2183,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J8" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="K8" t="str">
         <v>New</v>
@@ -2234,7 +2234,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J9" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
       </c>
       <c r="K9" t="str">
         <v>New</v>
@@ -2285,7 +2285,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J10" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K10" t="str">
         <v>New</v>
@@ -2336,7 +2336,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J11" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K11" t="str">
         <v>New</v>
@@ -2387,7 +2387,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J12" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K12" t="str">
         <v>New</v>
@@ -2438,7 +2438,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J13" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K13" t="str">
         <v>New</v>
@@ -2489,7 +2489,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J14" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K14" t="str">
         <v>New</v>
@@ -2540,7 +2540,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J15" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K15" t="str">
         <v>New</v>
@@ -2591,7 +2591,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J16" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K16" t="str">
         <v>New</v>
@@ -2642,7 +2642,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J17" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K17" t="str">
         <v>New</v>
@@ -2693,7 +2693,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J18" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K18" t="str">
         <v>New</v>
@@ -2744,7 +2744,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J19" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K19" t="str">
         <v>New</v>
@@ -2795,7 +2795,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J20" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K20" t="str">
         <v>New</v>
@@ -2846,7 +2846,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J21" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K21" t="str">
         <v>New</v>
@@ -2897,7 +2897,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J22" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K22" t="str">
         <v>New</v>
@@ -2948,7 +2948,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J23" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K23" t="str">
         <v>New</v>
@@ -2999,7 +2999,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J24" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K24" t="str">
         <v>New</v>
@@ -3050,7 +3050,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J25" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
       </c>
       <c r="K25" t="str">
         <v>New</v>

</xml_diff>

<commit_message>
CI Reports [2026-06-29 18:58]: ActionQueue — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/ActionQueue.xlsx
+++ b/Test Execution Report_Git/Feature Reports/ActionQueue.xlsx
@@ -500,7 +500,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K2" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('h1').filter({ hasText: 'Action Queue' }) Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('h1').filter({ hasText: 'Action Queue' })</v>
       </c>
       <c r="L2" t="str">
         <v>FAIL</v>
@@ -550,7 +550,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K3" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('p:has-text("Total Actions")').locator('..').locator('h3') Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('p:has-text("Total Actions")').locator('..'</v>
       </c>
       <c r="L3" t="str">
         <v>FAIL</v>
@@ -600,7 +600,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K4" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>Error: expect(received).toBeTruthy() Received: false</v>
       </c>
       <c r="L4" t="str">
         <v>FAIL</v>
@@ -650,7 +650,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K5" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for getByPlaceholder('Search actions...')</v>
       </c>
       <c r="L5" t="str">
         <v>FAIL</v>
@@ -700,7 +700,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K6" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for getByPlaceholder('Search actions...')</v>
       </c>
       <c r="L6" t="str">
         <v>FAIL</v>
@@ -750,7 +750,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K7" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>Error: expect(locator).toBeVisible() failed Locator: getByRole('button', { name: /EXPORT/i }) Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for getByRole('button', { name: /EXPORT/i })</v>
       </c>
       <c r="L7" t="str">
         <v>FAIL</v>
@@ -800,7 +800,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K8" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>TimeoutError: locator.textContent: Timeout 15000ms exceeded. Call log: - waiting for locator('text=/Page \\d+ of \\d+/')</v>
       </c>
       <c r="L8" t="str">
         <v>FAIL</v>
@@ -900,7 +900,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K10" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('[title="Perform Action"]').first()</v>
       </c>
       <c r="L10" t="str">
         <v>FAIL</v>
@@ -950,7 +950,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K11" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('text=Project Information').first() Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('text=Project Information').first()</v>
       </c>
       <c r="L11" t="str">
         <v>FAIL</v>
@@ -1050,7 +1050,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K13" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /TIMELINE/i })</v>
       </c>
       <c r="L13" t="str">
         <v>FAIL</v>
@@ -1100,7 +1100,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K14" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="L14" t="str">
         <v>FAIL</v>
@@ -1150,7 +1150,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K15" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="L15" t="str">
         <v>FAIL</v>
@@ -1200,7 +1200,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K16" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="L16" t="str">
         <v>FAIL</v>
@@ -1250,7 +1250,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K17" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="L17" t="str">
         <v>FAIL</v>
@@ -1300,7 +1300,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K18" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="L18" t="str">
         <v>FAIL</v>
@@ -1350,7 +1350,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K19" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="L19" t="str">
         <v>FAIL</v>
@@ -1400,7 +1400,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K20" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="L20" t="str">
         <v>FAIL</v>
@@ -1450,7 +1450,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K21" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="L21" t="str">
         <v>FAIL</v>
@@ -1500,7 +1500,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K22" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="L22" t="str">
         <v>FAIL</v>
@@ -1550,7 +1550,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K23" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /REOPEN/i })</v>
       </c>
       <c r="L23" t="str">
         <v>FAIL</v>
@@ -1600,7 +1600,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K24" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /REOPEN/i })</v>
       </c>
       <c r="L24" t="str">
         <v>FAIL</v>
@@ -1650,7 +1650,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K25" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /REOPEN/i })</v>
       </c>
       <c r="L25" t="str">
         <v>FAIL</v>
@@ -1700,7 +1700,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K26" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /REOPEN/i })</v>
       </c>
       <c r="L26" t="str">
         <v>FAIL</v>
@@ -1750,7 +1750,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K27" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /BACK/i })</v>
       </c>
       <c r="L27" t="str">
         <v>FAIL</v>
@@ -1877,7 +1877,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J2" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('h1').filter({ hasText: 'Action Queue' }) Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('h1').filter({ hasText: 'Action Queue' })</v>
       </c>
       <c r="K2" t="str">
         <v>New</v>
@@ -1928,7 +1928,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J3" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('p:has-text("Total Actions")').locator('..').locator('h3') Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('p:has-text("Total Actions")').locator('..'</v>
       </c>
       <c r="K3" t="str">
         <v>New</v>
@@ -1979,7 +1979,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J4" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>Error: expect(received).toBeTruthy() Received: false</v>
       </c>
       <c r="K4" t="str">
         <v>New</v>
@@ -2030,7 +2030,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J5" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for getByPlaceholder('Search actions...')</v>
       </c>
       <c r="K5" t="str">
         <v>New</v>
@@ -2081,7 +2081,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J6" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for getByPlaceholder('Search actions...')</v>
       </c>
       <c r="K6" t="str">
         <v>New</v>
@@ -2132,7 +2132,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J7" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>Error: expect(locator).toBeVisible() failed Locator: getByRole('button', { name: /EXPORT/i }) Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for getByRole('button', { name: /EXPORT/i })</v>
       </c>
       <c r="K7" t="str">
         <v>New</v>
@@ -2183,7 +2183,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J8" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>TimeoutError: locator.textContent: Timeout 15000ms exceeded. Call log: - waiting for locator('text=/Page \\d+ of \\d+/')</v>
       </c>
       <c r="K8" t="str">
         <v>New</v>
@@ -2234,7 +2234,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J9" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1').filter({ hasText: 'Action Queue' }) to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('[title="Perform Action"]').first()</v>
       </c>
       <c r="K9" t="str">
         <v>New</v>
@@ -2285,7 +2285,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J10" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('text=Project Information').first() Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('text=Project Information').first()</v>
       </c>
       <c r="K10" t="str">
         <v>New</v>
@@ -2336,7 +2336,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J11" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /TIMELINE/i })</v>
       </c>
       <c r="K11" t="str">
         <v>New</v>
@@ -2387,7 +2387,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J12" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="K12" t="str">
         <v>New</v>
@@ -2438,7 +2438,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J13" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="K13" t="str">
         <v>New</v>
@@ -2489,7 +2489,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J14" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="K14" t="str">
         <v>New</v>
@@ -2540,7 +2540,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J15" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="K15" t="str">
         <v>New</v>
@@ -2591,7 +2591,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J16" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="K16" t="str">
         <v>New</v>
@@ -2642,7 +2642,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J17" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="K17" t="str">
         <v>New</v>
@@ -2693,7 +2693,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J18" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="K18" t="str">
         <v>New</v>
@@ -2744,7 +2744,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J19" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="K19" t="str">
         <v>New</v>
@@ -2795,7 +2795,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J20" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /APPROVE/i })</v>
       </c>
       <c r="K20" t="str">
         <v>New</v>
@@ -2846,7 +2846,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J21" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /REOPEN/i })</v>
       </c>
       <c r="K21" t="str">
         <v>New</v>
@@ -2897,7 +2897,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J22" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /REOPEN/i })</v>
       </c>
       <c r="K22" t="str">
         <v>New</v>
@@ -2948,7 +2948,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J23" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /REOPEN/i })</v>
       </c>
       <c r="K23" t="str">
         <v>New</v>
@@ -2999,7 +2999,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J24" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /REOPEN/i })</v>
       </c>
       <c r="K24" t="str">
         <v>New</v>
@@ -3050,7 +3050,7 @@
         <v>All Playwright assertions pass</v>
       </c>
       <c r="J25" t="str">
-        <v>TimeoutError: locator.waitFor: Timeout 15000ms exceeded. Call log: - waiting for locator('h1') to be visible</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /BACK/i })</v>
       </c>
       <c r="K25" t="str">
         <v>New</v>

</xml_diff>

<commit_message>
Regression [Nightly 2026-06-30 20:17]: all — reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/ActionQueue.xlsx
+++ b/Test Execution Report_Git/Feature Reports/ActionQueue.xlsx
@@ -509,13 +509,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N2" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O2" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P2" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="3">
@@ -559,13 +559,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N3" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O3" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P3" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="4">
@@ -609,13 +609,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N4" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O4" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P4" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="5">
@@ -659,13 +659,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N5" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O5" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P5" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="6">
@@ -709,13 +709,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N6" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O6" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P6" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="7">
@@ -759,13 +759,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N7" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O7" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P7" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="8">
@@ -809,13 +809,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N8" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O8" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P8" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="9">
@@ -859,13 +859,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N9" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O9" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P9" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="10">
@@ -909,13 +909,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N10" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O10" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P10" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="11">
@@ -959,13 +959,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N11" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O11" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P11" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="12">
@@ -1009,13 +1009,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N12" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O12" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P12" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="13">
@@ -1059,13 +1059,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N13" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O13" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P13" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="14">
@@ -1109,13 +1109,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N14" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O14" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P14" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="15">
@@ -1159,13 +1159,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N15" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O15" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P15" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="16">
@@ -1209,13 +1209,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N16" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O16" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P16" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="17">
@@ -1259,13 +1259,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N17" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O17" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P17" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="18">
@@ -1309,13 +1309,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N18" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O18" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P18" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="19">
@@ -1359,13 +1359,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N19" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O19" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P19" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="20">
@@ -1409,13 +1409,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N20" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O20" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P20" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="21">
@@ -1459,13 +1459,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N21" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O21" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P21" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="22">
@@ -1509,13 +1509,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N22" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O22" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P22" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="23">
@@ -1559,13 +1559,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N23" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O23" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P23" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="24">
@@ -1609,13 +1609,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N24" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O24" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P24" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="25">
@@ -1659,13 +1659,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N25" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O25" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P25" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="26">
@@ -1709,13 +1709,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N26" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O26" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P26" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="27">
@@ -1759,13 +1759,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N27" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O27" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P27" t="str">
-        <v>Regression run — 6/29/2026, 8:17:27 PM</v>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="28">
@@ -1809,13 +1809,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N28" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O28" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P28" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="29">
@@ -1859,13 +1859,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N29" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O29" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P29" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="30">
@@ -1909,13 +1909,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N30" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O30" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P30" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="31">
@@ -1959,13 +1959,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N31" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O31" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P31" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="32">
@@ -2009,13 +2009,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N32" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O32" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P32" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="33">
@@ -2059,13 +2059,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N33" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O33" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P33" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="34">
@@ -2109,13 +2109,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N34" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O34" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P34" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="35">
@@ -2159,13 +2159,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N35" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O35" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P35" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="36">
@@ -2209,13 +2209,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N36" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O36" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P36" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="37">
@@ -2259,13 +2259,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N37" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O37" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P37" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="38">
@@ -2309,13 +2309,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N38" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O38" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P38" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="39">
@@ -2359,13 +2359,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N39" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O39" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P39" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="40">
@@ -2409,13 +2409,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N40" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O40" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P40" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="41">
@@ -2459,13 +2459,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N41" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O41" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P41" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="42">
@@ -2509,13 +2509,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N42" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O42" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P42" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="43">
@@ -2559,13 +2559,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N43" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O43" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P43" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="44">
@@ -2609,13 +2609,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N44" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O44" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P44" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="45">
@@ -2659,13 +2659,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N45" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O45" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P45" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="46">
@@ -2709,13 +2709,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N46" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O46" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P46" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="47">
@@ -2759,13 +2759,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N47" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O47" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P47" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="48">
@@ -2809,13 +2809,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N48" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O48" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P48" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="49">
@@ -2859,13 +2859,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N49" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O49" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P49" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="50">
@@ -2900,7 +2900,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K50" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L50" t="str">
         <v>PASS</v>
@@ -2909,13 +2909,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N50" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O50" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P50" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="51">
@@ -2959,13 +2959,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N51" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O51" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P51" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="52">
@@ -3000,22 +3000,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K52" t="str">
-        <v>Error: expect(locator).toBeVisible() failed Locator: locator('#btnOverview') Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#btnOverview')</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L52" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M52" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N52" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O52" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P52" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="53">
@@ -3059,13 +3059,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N53" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O53" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P53" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="54">
@@ -3109,13 +3109,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N54" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O54" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P54" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="55">
@@ -3150,7 +3150,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K55" t="str">
-        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-06-30" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-07-01" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
       </c>
       <c r="L55" t="str">
         <v>FAIL</v>
@@ -3159,13 +3159,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N55" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O55" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P55" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="56">
@@ -3200,7 +3200,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K56" t="str">
-        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-06-30" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-07-01" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
       </c>
       <c r="L56" t="str">
         <v>FAIL</v>
@@ -3209,13 +3209,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N56" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O56" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P56" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="57">
@@ -3250,7 +3250,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K57" t="str">
-        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-06-30" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-07-01" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
       </c>
       <c r="L57" t="str">
         <v>FAIL</v>
@@ -3259,13 +3259,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N57" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O57" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P57" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="58">
@@ -3300,7 +3300,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K58" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L58" t="str">
         <v>PASS</v>
@@ -3309,13 +3309,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N58" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O58" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P58" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="59">
@@ -3350,7 +3350,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K59" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L59" t="str">
         <v>PASS</v>
@@ -3359,13 +3359,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N59" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O59" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P59" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="60">
@@ -3400,7 +3400,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K60" t="str">
-        <v>Error: expect(locator).toBeVisible() failed Locator: locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout: 5000ms Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('a[href="/Ticket/Index"]').first() 14 × locator resolved to &lt;a data-id="4" tab</v>
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout: 5000ms Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('a[href="/Ticket/Index"]').first() 13 × locator resolved to &lt;a data-id="4" tab</v>
       </c>
       <c r="L60" t="str">
         <v>FAIL</v>
@@ -3409,13 +3409,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N60" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O60" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P60" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="61">
@@ -3459,13 +3459,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N61" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O61" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P61" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="62">
@@ -3500,7 +3500,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K62" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L62" t="str">
         <v>PASS</v>
@@ -3509,13 +3509,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N62" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O62" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P62" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="63">
@@ -3550,7 +3550,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K63" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L63" t="str">
         <v>PASS</v>
@@ -3559,13 +3559,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N63" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O63" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P63" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="64">
@@ -3600,7 +3600,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K64" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L64" t="str">
         <v>PASS</v>
@@ -3609,13 +3609,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N64" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O64" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P64" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="65">
@@ -3650,7 +3650,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K65" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L65" t="str">
         <v>PASS</v>
@@ -3659,13 +3659,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N65" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O65" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P65" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="66">
@@ -3700,7 +3700,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K66" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L66" t="str">
         <v>PASS</v>
@@ -3709,13 +3709,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N66" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O66" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P66" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="67">
@@ -3750,7 +3750,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K67" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L67" t="str">
         <v>PASS</v>
@@ -3759,13 +3759,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N67" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O67" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P67" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="68">
@@ -3800,7 +3800,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K68" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L68" t="str">
         <v>PASS</v>
@@ -3809,13 +3809,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N68" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O68" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P68" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="69">
@@ -3850,7 +3850,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K69" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L69" t="str">
         <v>PASS</v>
@@ -3859,13 +3859,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N69" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O69" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P69" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="70">
@@ -3900,7 +3900,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K70" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L70" t="str">
         <v>PASS</v>
@@ -3909,13 +3909,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N70" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O70" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P70" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="71">
@@ -3950,7 +3950,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K71" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L71" t="str">
         <v>PASS</v>
@@ -3959,13 +3959,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N71" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O71" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P71" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="72">
@@ -4000,7 +4000,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K72" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L72" t="str">
         <v>PASS</v>
@@ -4009,13 +4009,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N72" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O72" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P72" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="73">
@@ -4050,7 +4050,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K73" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L73" t="str">
         <v>PASS</v>
@@ -4059,13 +4059,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N73" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O73" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P73" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="74">
@@ -4100,7 +4100,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K74" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L74" t="str">
         <v>PASS</v>
@@ -4109,13 +4109,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N74" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O74" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P74" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="75">
@@ -4150,7 +4150,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K75" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L75" t="str">
         <v>PASS</v>
@@ -4159,13 +4159,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N75" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O75" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P75" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="76">
@@ -4200,7 +4200,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K76" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L76" t="str">
         <v>PASS</v>
@@ -4209,13 +4209,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N76" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O76" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P76" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="77">
@@ -4250,7 +4250,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K77" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L77" t="str">
         <v>PASS</v>
@@ -4259,13 +4259,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N77" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O77" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P77" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="78">
@@ -4300,7 +4300,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K78" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L78" t="str">
         <v>PASS</v>
@@ -4309,13 +4309,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N78" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O78" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P78" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="79">
@@ -4350,7 +4350,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K79" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L79" t="str">
         <v>PASS</v>
@@ -4359,13 +4359,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N79" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O79" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P79" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="80">
@@ -4400,7 +4400,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K80" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L80" t="str">
         <v>PASS</v>
@@ -4409,13 +4409,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N80" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O80" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P80" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="81">
@@ -4450,7 +4450,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K81" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L81" t="str">
         <v>PASS</v>
@@ -4459,13 +4459,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N81" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O81" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P81" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="82">
@@ -4500,7 +4500,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K82" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L82" t="str">
         <v>PASS</v>
@@ -4509,13 +4509,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N82" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O82" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P82" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="83">
@@ -4550,7 +4550,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K83" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L83" t="str">
         <v>PASS</v>
@@ -4559,13 +4559,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N83" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O83" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P83" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="84">
@@ -4600,7 +4600,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K84" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Test passed via Playwright automation</v>
       </c>
       <c r="L84" t="str">
         <v>PASS</v>
@@ -4609,13 +4609,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N84" t="str">
-        <v>29 Jun 2026</v>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O84" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P84" t="str">
-        <v/>
+        <v>Regression run — 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
   </sheetData>
@@ -7178,7 +7178,7 @@
         <v>Error: expect(locator).toBeVisible() failed Locator: locator('#btnOverview') Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#btnOverview')</v>
       </c>
       <c r="K50" t="str">
-        <v>New</v>
+        <v>Fixed</v>
       </c>
       <c r="L50" t="str">
         <v>Playwright Automation</v>
@@ -7187,13 +7187,13 @@
         <v>29 Jun 2026</v>
       </c>
       <c r="N50" t="str">
-        <v/>
+        <v>30 Jun 2026</v>
       </c>
       <c r="O50" t="str">
-        <v>Fail</v>
+        <v>Pass</v>
       </c>
       <c r="P50" t="str">
-        <v/>
+        <v>Fixed — verified in Playwright regression 6/30/2026, 8:17:21 PM</v>
       </c>
     </row>
     <row r="51" xml:space="preserve">

</xml_diff>

<commit_message>
Regression [Nightly 2026-07-02 19:49]: all — reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/ActionQueue.xlsx
+++ b/Test Execution Report_Git/Feature Reports/ActionQueue.xlsx
@@ -500,7 +500,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K2" t="str">
-        <v>Error: expect(locator).toBeVisible() failed Locator: locator('text=7 Pending Actions') Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('text=7 Pending Actions')</v>
+        <v>TypeError: aq.navigateToActionQueue is not a function</v>
       </c>
       <c r="L2" t="str">
         <v>FAIL</v>
@@ -509,13 +509,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N2" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O2" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P2" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="3">
@@ -550,22 +550,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K3" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueue is not a function</v>
       </c>
       <c r="L3" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M3" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N3" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O3" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P3" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="4">
@@ -600,22 +600,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K4" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueue is not a function</v>
       </c>
       <c r="L4" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M4" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N4" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O4" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P4" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="5">
@@ -650,7 +650,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K5" t="str">
-        <v>Error: expect(received).toBeGreaterThanOrEqual(expected) Expected: &gt;= 1 Received: 0</v>
+        <v>TypeError: aq.navigateToActionQueue is not a function</v>
       </c>
       <c r="L5" t="str">
         <v>FAIL</v>
@@ -659,13 +659,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N5" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O5" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P5" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="6">
@@ -700,22 +700,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K6" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueue is not a function</v>
       </c>
       <c r="L6" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M6" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N6" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O6" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P6" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="7">
@@ -750,22 +750,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K7" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueue is not a function</v>
       </c>
       <c r="L7" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M7" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N7" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O7" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P7" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="8">
@@ -800,22 +800,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K8" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueue is not a function</v>
       </c>
       <c r="L8" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M8" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N8" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O8" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P8" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="9">
@@ -859,13 +859,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N9" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O9" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P9" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="10">
@@ -900,22 +900,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K10" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueue is not a function</v>
       </c>
       <c r="L10" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M10" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N10" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O10" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P10" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="11">
@@ -950,22 +950,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K11" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L11" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M11" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N11" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O11" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P11" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="12">
@@ -1009,13 +1009,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N12" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O12" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P12" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="13">
@@ -1050,22 +1050,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K13" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L13" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M13" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N13" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O13" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P13" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="14">
@@ -1100,22 +1100,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K14" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L14" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M14" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N14" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O14" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P14" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="15">
@@ -1150,22 +1150,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K15" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L15" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M15" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N15" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O15" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P15" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="16">
@@ -1200,22 +1200,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K16" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L16" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M16" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N16" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O16" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P16" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="17">
@@ -1250,22 +1250,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K17" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L17" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M17" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N17" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O17" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P17" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="18">
@@ -1300,7 +1300,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K18" t="str">
-        <v>Error: expect(received).toBeTruthy() Received: false</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L18" t="str">
         <v>FAIL</v>
@@ -1309,13 +1309,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N18" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O18" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P18" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="19">
@@ -1350,22 +1350,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K19" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L19" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M19" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N19" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O19" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P19" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="20">
@@ -1400,22 +1400,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K20" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L20" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M20" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N20" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O20" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P20" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="21">
@@ -1450,22 +1450,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K21" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L21" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M21" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N21" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O21" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P21" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="22">
@@ -1500,22 +1500,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K22" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L22" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M22" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N22" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O22" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P22" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="23">
@@ -1550,22 +1550,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K23" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L23" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M23" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N23" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O23" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P23" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="24">
@@ -1600,22 +1600,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K24" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L24" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M24" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N24" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O24" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P24" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="25">
@@ -1650,22 +1650,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K25" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L25" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M25" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N25" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O25" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P25" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="26">
@@ -1700,22 +1700,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K26" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L26" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M26" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N26" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O26" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P26" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="27">
@@ -1750,7 +1750,7 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K27" t="str">
-        <v>Error: expect(received).not.toMatch(expected) Expected pattern: not /ActionQueueDetails/ Received string: "http://customerportal.dev-ts.online/Ticket/ActionQueueDetails/1345"</v>
+        <v>TypeError: aq.navigateToActionQueueDetails is not a function</v>
       </c>
       <c r="L27" t="str">
         <v>FAIL</v>
@@ -1759,13 +1759,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N27" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O27" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P27" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="28">
@@ -1809,13 +1809,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N28" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O28" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P28" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="29">
@@ -1850,22 +1850,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K29" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L29" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M29" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N29" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O29" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P29" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="30">
@@ -1909,13 +1909,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N30" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O30" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P30" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="31">
@@ -1950,22 +1950,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K31" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L31" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M31" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N31" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O31" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P31" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="32">
@@ -2000,22 +2000,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K32" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L32" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M32" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N32" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O32" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P32" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="33">
@@ -2059,13 +2059,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N33" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O33" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P33" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="34">
@@ -2109,13 +2109,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N34" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O34" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P34" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="35">
@@ -2150,22 +2150,22 @@
         <v>Test assertions pass per spec definition</v>
       </c>
       <c r="K35" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L35" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M35" t="str">
         <v>Playwright Automation</v>
       </c>
       <c r="N35" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O35" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P35" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="36">
@@ -2209,13 +2209,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N36" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O36" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P36" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="37">
@@ -2259,13 +2259,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N37" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O37" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P37" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="38">
@@ -2309,13 +2309,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N38" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O38" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P38" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="39">
@@ -2359,13 +2359,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N39" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O39" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P39" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="40">
@@ -2409,13 +2409,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N40" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O40" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P40" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="41">
@@ -2459,13 +2459,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N41" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O41" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P41" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="42">
@@ -2509,13 +2509,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N42" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O42" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P42" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="43">
@@ -2559,13 +2559,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N43" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O43" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P43" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="44">
@@ -2609,13 +2609,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N44" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O44" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P44" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="45">
@@ -2659,13 +2659,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N45" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O45" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P45" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="46">
@@ -2709,13 +2709,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N46" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O46" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P46" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="47">
@@ -2759,13 +2759,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N47" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O47" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P47" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="48">
@@ -2809,13 +2809,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N48" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O48" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P48" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="49">
@@ -2859,13 +2859,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N49" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O49" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P49" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="50">
@@ -2909,13 +2909,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N50" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O50" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P50" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="51">
@@ -2959,13 +2959,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N51" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O51" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P51" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="52">
@@ -3009,13 +3009,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N52" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O52" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P52" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="53">
@@ -3059,13 +3059,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N53" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O53" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P53" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="54">
@@ -3109,13 +3109,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N54" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O54" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P54" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="55">
@@ -3159,13 +3159,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N55" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O55" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P55" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="56">
@@ -3209,13 +3209,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N56" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O56" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P56" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="57">
@@ -3259,13 +3259,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N57" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O57" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P57" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="58">
@@ -3309,13 +3309,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N58" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O58" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P58" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="59">
@@ -3359,13 +3359,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N59" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O59" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P59" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="60">
@@ -3409,13 +3409,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N60" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O60" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P60" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="61">
@@ -3459,13 +3459,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N61" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O61" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P61" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="62">
@@ -3509,13 +3509,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N62" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O62" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P62" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="63">
@@ -3559,13 +3559,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N63" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O63" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P63" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="64">
@@ -3609,13 +3609,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N64" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O64" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P64" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="65">
@@ -3659,13 +3659,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N65" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O65" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P65" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="66">
@@ -3709,13 +3709,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N66" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O66" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P66" t="str">
-        <v/>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="67">
@@ -3759,13 +3759,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N67" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O67" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P67" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="68">
@@ -3809,13 +3809,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N68" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O68" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P68" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="69">
@@ -3859,13 +3859,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N69" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O69" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P69" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="70">
@@ -3909,13 +3909,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N70" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O70" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P70" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="71">
@@ -3959,13 +3959,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N71" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O71" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P71" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="72">
@@ -4009,13 +4009,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N72" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O72" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P72" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="73">
@@ -4059,13 +4059,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N73" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O73" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P73" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="74">
@@ -4109,13 +4109,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N74" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O74" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P74" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="75">
@@ -4159,13 +4159,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N75" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O75" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P75" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="76">
@@ -4209,13 +4209,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N76" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O76" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P76" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="77">
@@ -4259,13 +4259,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N77" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O77" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P77" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="78">
@@ -4309,13 +4309,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N78" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O78" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P78" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="79">
@@ -4359,13 +4359,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N79" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O79" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P79" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="80">
@@ -4409,13 +4409,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N80" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O80" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P80" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="81">
@@ -4459,13 +4459,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N81" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O81" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P81" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="82">
@@ -4509,13 +4509,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N82" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O82" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P82" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="83">
@@ -4559,13 +4559,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N83" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O83" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P83" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="84">
@@ -4609,13 +4609,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N84" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O84" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P84" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="85">
@@ -4659,13 +4659,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N85" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O85" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P85" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="86">
@@ -4709,13 +4709,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N86" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O86" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P86" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="87">
@@ -4759,13 +4759,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N87" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O87" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P87" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="88">
@@ -4809,13 +4809,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N88" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O88" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P88" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="89">
@@ -4859,13 +4859,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N89" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O89" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P89" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="90">
@@ -4909,13 +4909,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N90" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O90" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P90" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="91">
@@ -4959,13 +4959,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N91" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O91" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P91" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="92">
@@ -5009,13 +5009,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N92" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O92" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P92" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="93">
@@ -5059,13 +5059,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N93" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O93" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P93" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="94">
@@ -5109,13 +5109,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N94" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O94" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P94" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="95">
@@ -5159,13 +5159,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N95" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O95" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P95" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="96">
@@ -5209,13 +5209,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N96" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O96" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P96" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="97">
@@ -5259,13 +5259,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N97" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O97" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P97" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="98">
@@ -5309,13 +5309,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N98" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O98" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P98" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="99">
@@ -5359,13 +5359,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N99" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O99" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P99" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="100">
@@ -5409,13 +5409,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N100" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O100" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P100" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="101">
@@ -5459,13 +5459,13 @@
         <v>Playwright Automation</v>
       </c>
       <c r="N101" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O101" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="P101" t="str">
-        <v>Regression run — 7/1/2026, 8:22:09 PM</v>
+        <v>Regression run — 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
   </sheetData>
@@ -6048,13 +6048,13 @@
         <v>29 Jun 2026</v>
       </c>
       <c r="N11" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O11" t="str">
         <v>Pass</v>
       </c>
       <c r="P11" t="str">
-        <v>Fixed — verified in Playwright regression 7/1/2026, 8:22:09 PM</v>
+        <v>Fixed — verified in Playwright regression 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -8037,13 +8037,13 @@
         <v>29 Jun 2026</v>
       </c>
       <c r="N50" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O50" t="str">
         <v>Pass</v>
       </c>
       <c r="P50" t="str">
-        <v>Fixed — verified in Playwright regression 7/1/2026, 8:22:09 PM</v>
+        <v>Fixed — verified in Playwright regression 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="51" xml:space="preserve">
@@ -8394,13 +8394,13 @@
         <v>29 Jun 2026</v>
       </c>
       <c r="N57" t="str">
-        <v>01 Jul 2026</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O57" t="str">
         <v>Pass</v>
       </c>
       <c r="P57" t="str">
-        <v>Fixed — verified in Playwright regression 7/1/2026, 8:22:09 PM</v>
+        <v>Fixed — verified in Playwright regression 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="58" xml:space="preserve">
@@ -8437,7 +8437,7 @@
         <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="K58" t="str">
-        <v>New</v>
+        <v>Fixed</v>
       </c>
       <c r="L58" t="str">
         <v>Playwright Automation</v>
@@ -8446,13 +8446,13 @@
         <v>01 Jul 2026</v>
       </c>
       <c r="N58" t="str">
-        <v/>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O58" t="str">
-        <v>Fail</v>
+        <v>Pass</v>
       </c>
       <c r="P58" t="str">
-        <v/>
+        <v>Fixed — verified in Playwright regression 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="59" xml:space="preserve">
@@ -8541,7 +8541,7 @@
         <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="K60" t="str">
-        <v>New</v>
+        <v>Fixed</v>
       </c>
       <c r="L60" t="str">
         <v>Playwright Automation</v>
@@ -8550,13 +8550,13 @@
         <v>01 Jul 2026</v>
       </c>
       <c r="N60" t="str">
-        <v/>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O60" t="str">
-        <v>Fail</v>
+        <v>Pass</v>
       </c>
       <c r="P60" t="str">
-        <v/>
+        <v>Fixed — verified in Playwright regression 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="61" xml:space="preserve">
@@ -8593,7 +8593,7 @@
         <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="K61" t="str">
-        <v>New</v>
+        <v>Fixed</v>
       </c>
       <c r="L61" t="str">
         <v>Playwright Automation</v>
@@ -8602,13 +8602,13 @@
         <v>01 Jul 2026</v>
       </c>
       <c r="N61" t="str">
-        <v/>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O61" t="str">
-        <v>Fail</v>
+        <v>Pass</v>
       </c>
       <c r="P61" t="str">
-        <v/>
+        <v>Fixed — verified in Playwright regression 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="62" xml:space="preserve">
@@ -8645,7 +8645,7 @@
         <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="K62" t="str">
-        <v>New</v>
+        <v>Fixed</v>
       </c>
       <c r="L62" t="str">
         <v>Playwright Automation</v>
@@ -8654,13 +8654,13 @@
         <v>01 Jul 2026</v>
       </c>
       <c r="N62" t="str">
-        <v/>
+        <v>02 Jul 2026</v>
       </c>
       <c r="O62" t="str">
-        <v>Fail</v>
+        <v>Pass</v>
       </c>
       <c r="P62" t="str">
-        <v/>
+        <v>Fixed — verified in Playwright regression 7/2/2026, 7:49:54 PM</v>
       </c>
     </row>
     <row r="63" xml:space="preserve">

</xml_diff>